<commit_message>
clarifying stats being tracked in overview
</commit_message>
<xml_diff>
--- a/UCLStats25-26.xlsx
+++ b/UCLStats25-26.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johntran/VSCode/VSCode for ACM/mpacmphase2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE72912B-4ED0-1249-8599-8AAD8B8DA42B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8ACBB9-78F2-5243-B847-7C3EBD1F266C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="900" windowWidth="28040" windowHeight="17100" xr2:uid="{802A0F31-8C0E-1546-A7F6-97F3B02C124B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -134,12 +134,6 @@
     <t>GamesPlayed</t>
   </si>
   <si>
-    <t>RedCards</t>
-  </si>
-  <si>
-    <t>YellowCards</t>
-  </si>
-  <si>
     <t>Goals</t>
   </si>
   <si>
@@ -155,9 +149,6 @@
     <t>Passes</t>
   </si>
   <si>
-    <t>Fouls</t>
-  </si>
-  <si>
     <t>SucessfulTackles</t>
   </si>
   <si>
@@ -168,6 +159,15 @@
   </si>
   <si>
     <t>AccuratePasses</t>
+  </si>
+  <si>
+    <t>GoalsConceded</t>
+  </si>
+  <si>
+    <t>FoulsCommitted</t>
+  </si>
+  <si>
+    <t>Tackles</t>
   </si>
 </sst>
 </file>
@@ -552,12 +552,12 @@
     <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
@@ -574,40 +574,40 @@
         <v>31</v>
       </c>
       <c r="E1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" t="s">
         <v>34</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>35</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>36</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1" t="s">
         <v>37</v>
       </c>
-      <c r="I1" t="s">
+      <c r="N1" t="s">
         <v>38</v>
-      </c>
-      <c r="J1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K1" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1" t="s">
-        <v>40</v>
-      </c>
-      <c r="M1" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" t="s">
-        <v>32</v>
       </c>
       <c r="O1" t="s">
         <v>41</v>
       </c>
       <c r="P1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -623,8 +623,11 @@
       <c r="D2">
         <v>7</v>
       </c>
+      <c r="N2">
+        <v>16</v>
+      </c>
       <c r="O2">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -643,6 +646,15 @@
       <c r="D3">
         <v>4</v>
       </c>
+      <c r="N3">
+        <v>10</v>
+      </c>
+      <c r="O3">
+        <v>6</v>
+      </c>
+      <c r="P3">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -657,12 +669,6 @@
       <c r="D4">
         <v>8</v>
       </c>
-      <c r="M4">
-        <v>2</v>
-      </c>
-      <c r="N4">
-        <v>1</v>
-      </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -677,12 +683,6 @@
       <c r="D5">
         <v>9</v>
       </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -697,12 +697,6 @@
       <c r="D6">
         <v>8</v>
       </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -717,12 +711,6 @@
       <c r="D7">
         <v>7</v>
       </c>
-      <c r="M7">
-        <v>1</v>
-      </c>
-      <c r="N7">
-        <v>0</v>
-      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -737,9 +725,6 @@
       <c r="D8">
         <v>2</v>
       </c>
-      <c r="M8">
-        <v>1</v>
-      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -754,9 +739,6 @@
       <c r="D9">
         <v>10</v>
       </c>
-      <c r="M9">
-        <v>2</v>
-      </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -771,12 +753,6 @@
       <c r="D10">
         <v>4</v>
       </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -791,12 +767,6 @@
       <c r="D11">
         <v>9</v>
       </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11">
-        <v>0</v>
-      </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -808,6 +778,9 @@
       <c r="C12" t="s">
         <v>27</v>
       </c>
+      <c r="D12">
+        <v>7</v>
+      </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -819,6 +792,18 @@
       <c r="C13" t="s">
         <v>27</v>
       </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -830,6 +815,9 @@
       <c r="C14" t="s">
         <v>27</v>
       </c>
+      <c r="D14">
+        <v>7</v>
+      </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -841,6 +829,9 @@
       <c r="C15" t="s">
         <v>27</v>
       </c>
+      <c r="D15">
+        <v>8</v>
+      </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -852,8 +843,11 @@
       <c r="C16" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D16">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -863,8 +857,11 @@
       <c r="C17" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D17">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -874,8 +871,11 @@
       <c r="C18" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -885,8 +885,11 @@
       <c r="C19" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D19">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -896,8 +899,11 @@
       <c r="C20" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D20">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -907,8 +913,11 @@
       <c r="C21" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -918,8 +927,11 @@
       <c r="C22" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D22">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -929,8 +941,11 @@
       <c r="C23" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D23">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -939,6 +954,9 @@
       </c>
       <c r="C24" t="s">
         <v>5</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>